<commit_message>
Hosting priced per environment set; environment model by broker size (in progress)
</commit_message>
<xml_diff>
--- a/docs/package/01_Sales/iNXT_BrokerVerse_ROI_Calculator.xlsx
+++ b/docs/package/01_Sales/iNXT_BrokerVerse_ROI_Calculator.xlsx
@@ -2986,19 +2986,19 @@
         </is>
       </c>
       <c r="B6" s="17" t="n">
-        <v>2066000</v>
+        <v>2264000</v>
       </c>
       <c r="C6" s="17" t="n">
-        <v>964800</v>
+        <v>1141800</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>995040</v>
+        <v>1172040</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>1026792</v>
+        <v>1203792</v>
       </c>
       <c r="F6" s="17" t="n">
-        <v>1060131.6</v>
+        <v>1237131.6</v>
       </c>
       <c r="G6" s="14">
         <f>SUM(B6:F6)</f>
@@ -3012,19 +3012,19 @@
         </is>
       </c>
       <c r="B7" s="17" t="n">
-        <v>2840000</v>
+        <v>3038000</v>
       </c>
       <c r="C7" s="17" t="n">
-        <v>657000</v>
+        <v>834000</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>671850</v>
+        <v>848850</v>
       </c>
       <c r="E7" s="17" t="n">
-        <v>687442.5</v>
+        <v>864442.5</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>703814.62</v>
+        <v>880814.62</v>
       </c>
       <c r="G7" s="14">
         <f>SUM(B7:F7)</f>
@@ -3038,19 +3038,19 @@
         </is>
       </c>
       <c r="B8" s="17" t="n">
-        <v>3356000</v>
+        <v>3564000</v>
       </c>
       <c r="C8" s="17" t="n">
-        <v>885000</v>
+        <v>1073000</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>912450</v>
+        <v>1100450</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>941272.5</v>
+        <v>1129272.5</v>
       </c>
       <c r="F8" s="17" t="n">
-        <v>971536.12</v>
+        <v>1159536.12</v>
       </c>
       <c r="G8" s="14">
         <f>SUM(B8:F8)</f>
@@ -3090,19 +3090,19 @@
         </is>
       </c>
       <c r="B10" s="17" t="n">
-        <v>4970000</v>
+        <v>5148000</v>
       </c>
       <c r="C10" s="17" t="n">
-        <v>2986800</v>
+        <v>3117800</v>
       </c>
       <c r="D10" s="17" t="n">
-        <v>3098940</v>
+        <v>3229940</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>3216687</v>
+        <v>3347687</v>
       </c>
       <c r="F10" s="17" t="n">
-        <v>3340321.35</v>
+        <v>3471321.35</v>
       </c>
       <c r="G10" s="14">
         <f>SUM(B10:F10)</f>
@@ -3116,19 +3116,19 @@
         </is>
       </c>
       <c r="B11" s="17" t="n">
-        <v>7814000</v>
+        <v>7992000</v>
       </c>
       <c r="C11" s="17" t="n">
-        <v>1839600</v>
+        <v>1970600</v>
       </c>
       <c r="D11" s="17" t="n">
-        <v>1894380</v>
+        <v>2025380</v>
       </c>
       <c r="E11" s="17" t="n">
-        <v>1951899</v>
+        <v>2082899</v>
       </c>
       <c r="F11" s="17" t="n">
-        <v>2012293.95</v>
+        <v>2143293.95</v>
       </c>
       <c r="G11" s="14">
         <f>SUM(B11:F11)</f>
@@ -3142,19 +3142,19 @@
         </is>
       </c>
       <c r="B12" s="17" t="n">
-        <v>8558000</v>
+        <v>8744000</v>
       </c>
       <c r="C12" s="17" t="n">
-        <v>2307600</v>
+        <v>2448600</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>2387580</v>
+        <v>2528580</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>2471559</v>
+        <v>2612559</v>
       </c>
       <c r="F12" s="17" t="n">
-        <v>2559736.95</v>
+        <v>2700736.95</v>
       </c>
       <c r="G12" s="14">
         <f>SUM(B12:F12)</f>
@@ -3194,19 +3194,19 @@
         </is>
       </c>
       <c r="B14" s="17" t="n">
-        <v>10828000</v>
+        <v>11372000</v>
       </c>
       <c r="C14" s="17" t="n">
-        <v>7417200</v>
+        <v>7875200</v>
       </c>
       <c r="D14" s="17" t="n">
-        <v>7720860</v>
+        <v>8178860</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>8039703</v>
+        <v>8497703</v>
       </c>
       <c r="F14" s="17" t="n">
-        <v>8374488.15</v>
+        <v>8832488.15</v>
       </c>
       <c r="G14" s="14">
         <f>SUM(B14:F14)</f>
@@ -3220,19 +3220,19 @@
         </is>
       </c>
       <c r="B15" s="17" t="n">
-        <v>18424000</v>
+        <v>18968000</v>
       </c>
       <c r="C15" s="17" t="n">
-        <v>4287600</v>
+        <v>4745600</v>
       </c>
       <c r="D15" s="17" t="n">
-        <v>4434780</v>
+        <v>4892780</v>
       </c>
       <c r="E15" s="17" t="n">
-        <v>4589319</v>
+        <v>5047319</v>
       </c>
       <c r="F15" s="17" t="n">
-        <v>4751584.95</v>
+        <v>5209584.95</v>
       </c>
       <c r="G15" s="14">
         <f>SUM(B15:F15)</f>
@@ -3246,19 +3246,19 @@
         </is>
       </c>
       <c r="B16" s="17" t="n">
-        <v>19564000</v>
+        <v>20064000</v>
       </c>
       <c r="C16" s="17" t="n">
-        <v>5172600</v>
+        <v>5590600</v>
       </c>
       <c r="D16" s="17" t="n">
-        <v>5367030</v>
+        <v>5785030</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>5571181.5</v>
+        <v>5989181.5</v>
       </c>
       <c r="F16" s="17" t="n">
-        <v>5785540.58</v>
+        <v>6203540.58</v>
       </c>
       <c r="G16" s="14">
         <f>SUM(B16:F16)</f>
@@ -3298,19 +3298,19 @@
         </is>
       </c>
       <c r="B18" s="17" t="n">
-        <v>20368000</v>
+        <v>20850000</v>
       </c>
       <c r="C18" s="17" t="n">
-        <v>15150000</v>
+        <v>15463000</v>
       </c>
       <c r="D18" s="17" t="n">
-        <v>15761100</v>
+        <v>16074100</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>16402755</v>
+        <v>16715755</v>
       </c>
       <c r="F18" s="17" t="n">
-        <v>17076492.75</v>
+        <v>17389492.75</v>
       </c>
       <c r="G18" s="14">
         <f>SUM(B18:F18)</f>
@@ -3324,19 +3324,19 @@
         </is>
       </c>
       <c r="B19" s="17" t="n">
-        <v>35428000</v>
+        <v>35910000</v>
       </c>
       <c r="C19" s="17" t="n">
-        <v>8802000</v>
+        <v>9115000</v>
       </c>
       <c r="D19" s="17" t="n">
-        <v>9095700</v>
+        <v>9408700</v>
       </c>
       <c r="E19" s="17" t="n">
-        <v>9404085</v>
+        <v>9717085</v>
       </c>
       <c r="F19" s="17" t="n">
-        <v>9727889.25</v>
+        <v>10040889.25</v>
       </c>
       <c r="G19" s="14">
         <f>SUM(B19:F19)</f>
@@ -3350,19 +3350,19 @@
         </is>
       </c>
       <c r="B20" s="17" t="n">
-        <v>37084000</v>
+        <v>37524000</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>10233000</v>
+        <v>10513000</v>
       </c>
       <c r="D20" s="17" t="n">
-        <v>10605450</v>
+        <v>10885450</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>10996522.5</v>
+        <v>11276522.5</v>
       </c>
       <c r="F20" s="17" t="n">
-        <v>11407148.62</v>
+        <v>11687148.62</v>
       </c>
       <c r="G20" s="14">
         <f>SUM(B20:F20)</f>

</xml_diff>